<commit_message>
AAB MOC draft 3: HAZID first and gospel; actions are the six approvals plus one per HAZID entry; H16 go-live gate added to the HAZID; MOC tool rule in the plan
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/AAB-HAZID-Register.xlsx
+++ b/AAB-HAZID-Register.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1574,6 +1574,73 @@
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="105" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>H16</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Change implemented out of order or untested before go-live</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Parts built by three parties go live out of step; flow never run in test mode; rigs not told how to acknowledge; deviation case not raised</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>The pilot starts on a route nobody has walked end to end</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Build order fixed in the plan; test mode proven on the CBM to OEM loop; HAZID and MOC precede the pilot; deviation case connected to the MOC</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Six-point go-live gate signed by the MOC owner: Rev 5 proven on the test records; scanner, register, acknowledgement page and AAB tab proven on the synthetic records; flow run in test mode; one advisory end to end on one rig in test mode with both TSLs and the chase; rig bulletin issued and office trained; deviation case open</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Dan</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>

</xml_diff>